<commit_message>
Refactorización: Teoría de la inf
Cambié de lugar todas las carpetas y me preparé para MC
</commit_message>
<xml_diff>
--- a/Teoría de la información/Canales.xlsx
+++ b/Teoría de la información/Canales.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repositories\Semestre-EneJun2026\Teoría de la información\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ran\Programas\GitHub\Repositorios\Semestre-EneJun2026\Teoría de la información\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04F5E0F7-5647-4DCB-A866-2359396FD640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D2AA9563-BBE5-4231-98B2-B4D59857FCAF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="23">
   <si>
     <t>M1</t>
   </si>
@@ -96,13 +95,32 @@
   </si>
   <si>
     <t>Probabilidad de que sea enviado</t>
+  </si>
+  <si>
+    <t>Esta matríz enlista la probabilidad de mandar una letra A y recibir una B</t>
+  </si>
+  <si>
+    <t>Esta matríz enlista la probabilidad de que salga cada cada letra en específico</t>
+  </si>
+  <si>
+    <t>Probabilidad total de error:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="2">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -203,10 +221,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -249,16 +268,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -293,7 +314,7 @@
         <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7350936D-E5CB-0339-932B-3F5003ED0A47}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{7350936D-E5CB-0339-932B-3F5003ED0A47}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -322,22 +343,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>172278</xdr:colOff>
+      <xdr:colOff>245165</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>19878</xdr:rowOff>
+      <xdr:rowOff>33130</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>619066</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>164105</xdr:rowOff>
+      <xdr:colOff>691954</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>5079</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5772B6C9-56AC-E841-7592-9B16F0AB9242}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{5772B6C9-56AC-E841-7592-9B16F0AB9242}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -353,8 +374,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5903843" y="2047461"/>
-          <a:ext cx="6012701" cy="1257409"/>
+          <a:off x="6460435" y="1954695"/>
+          <a:ext cx="6430145" cy="1177897"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -682,15 +703,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D151E52-2E79-4234-BFD9-0653B2E1C303}">
-  <dimension ref="B2:G21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:I24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
-    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:7" ht="15" customHeight="1"/>
+    <row r="3" spans="2:7" ht="27.6" customHeight="1">
       <c r="B3" s="12" t="s">
         <v>17</v>
       </c>
@@ -707,7 +728,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7">
       <c r="B4" s="10" t="s">
         <v>0</v>
       </c>
@@ -724,7 +745,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7">
       <c r="B5" s="10" t="s">
         <v>1</v>
       </c>
@@ -743,7 +764,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7">
       <c r="B6" s="10" t="s">
         <v>2</v>
       </c>
@@ -762,7 +783,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -775,7 +796,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -786,216 +807,227 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:7" s="18" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B11" s="16" t="s">
+    <row r="9" spans="2:7" s="16" customFormat="1"/>
+    <row r="11" spans="2:7">
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7">
+      <c r="B12" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+    </row>
+    <row r="13" spans="2:7">
+      <c r="B13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="4"/>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B13" s="4">
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="2:7">
+      <c r="B14" s="4">
         <v>0.4</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D14" s="5">
         <v>0.94</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E14" s="5">
         <v>0.04</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F14" s="5">
         <v>0.02</v>
-      </c>
-      <c r="G13" s="4">
-        <f>SUM(D13:F13)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B14" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="5">
-        <v>0.01</v>
-      </c>
-      <c r="E14" s="5">
-        <v>0.93</v>
-      </c>
-      <c r="F14" s="5">
-        <v>0.06</v>
       </c>
       <c r="G14" s="4">
         <f>SUM(D14:F14)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7">
       <c r="B15" s="4">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D15" s="5">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="E15" s="5">
-        <v>0.04</v>
+        <v>0.93</v>
       </c>
       <c r="F15" s="5">
-        <v>0.93</v>
+        <v>0.06</v>
       </c>
       <c r="G15" s="4">
         <f>SUM(D15:F15)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B16" s="17" t="s">
+    <row r="16" spans="2:7">
+      <c r="B16" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="5">
+        <v>0.03</v>
+      </c>
+      <c r="E16" s="5">
+        <v>0.04</v>
+      </c>
+      <c r="F16" s="5">
+        <v>0.93</v>
+      </c>
+      <c r="G16" s="4">
+        <f>SUM(D16:F16)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9">
+      <c r="B18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9">
+      <c r="B19" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B17" s="6" t="s">
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+    </row>
+    <row r="20" spans="2:9">
+      <c r="B20" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C20" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D20" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E20" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F20" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="8"/>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B18" s="8">
+      <c r="G20" s="8"/>
+      <c r="I20" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9">
+      <c r="B21" s="8"/>
+      <c r="C21" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="9">
+        <f>D14 * B14</f>
+        <v>0.376</v>
+      </c>
+      <c r="E21" s="9">
+        <f>E14 * B14</f>
+        <v>1.6E-2</v>
+      </c>
+      <c r="F21" s="9">
+        <f>F14 * B$14</f>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="G21" s="8">
+        <f>SUM(D21:F21)</f>
         <v>0.4</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="9">
-        <f>D13 * B13</f>
-        <v>0.376</v>
-      </c>
-      <c r="E18" s="9">
-        <f>E13 * B13</f>
-        <v>1.6E-2</v>
-      </c>
-      <c r="F18" s="9">
-        <f>F13 * B$13</f>
-        <v>8.0000000000000002E-3</v>
-      </c>
-      <c r="G18" s="8">
-        <f>SUM(D18:F18)</f>
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B19" s="8">
+      <c r="I21" s="19">
+        <f>SUM(E21, F21, D22, F22, D23, E23)</f>
+        <v>6.6000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9">
+      <c r="B22" s="8"/>
+      <c r="C22" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="9">
+        <f>D15 * B15</f>
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="E22" s="9">
+        <f>E15 * B15</f>
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="F22" s="9">
+        <f>F15 * B$15</f>
+        <v>0.03</v>
+      </c>
+      <c r="G22" s="8">
+        <f>SUM(D22:F22)</f>
         <v>0.5</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="9">
-        <f>D14 * B14</f>
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="E19" s="9">
-        <f>E14 * B14</f>
-        <v>0.46500000000000002</v>
-      </c>
-      <c r="F19" s="9">
-        <f>F14 * B$14</f>
-        <v>0.03</v>
-      </c>
-      <c r="G19" s="8">
-        <f>SUM(D19:F19)</f>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B20" s="8">
-        <v>0.1</v>
-      </c>
-      <c r="C20" s="7" t="s">
+    </row>
+    <row r="23" spans="2:9">
+      <c r="B23" s="8"/>
+      <c r="C23" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="9">
-        <f>D15 * B15</f>
+      <c r="D23" s="9">
+        <f>D16 * B16</f>
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="E20" s="9">
-        <f>E15 * B15</f>
+      <c r="E23" s="9">
+        <f>E16 * B16</f>
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="F20" s="9">
-        <f>F15 * B$15</f>
+      <c r="F23" s="9">
+        <f>F16 * B$16</f>
         <v>9.3000000000000013E-2</v>
       </c>
-      <c r="G20" s="8">
-        <f>SUM(D20:F20)</f>
+      <c r="G23" s="8">
+        <f>SUM(D23:F23)</f>
         <v>0.10000000000000002</v>
       </c>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="D21">
-        <f>SUM(D18:D20)</f>
+    <row r="24" spans="2:9">
+      <c r="D24">
+        <f>SUM(D21:D23)</f>
         <v>0.38400000000000001</v>
       </c>
-      <c r="E21">
-        <f>SUM(E18:E20)</f>
+      <c r="E24">
+        <f>SUM(E21:E23)</f>
         <v>0.48500000000000004</v>
       </c>
-      <c r="F21">
-        <f>SUM(F18:F20)</f>
+      <c r="F24">
+        <f>SUM(F21:F23)</f>
         <v>0.13100000000000001</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B19:G19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>